<commit_message>
Show category token cost breakdowns
</commit_message>
<xml_diff>
--- a/artifacts/cache-hit-budget.xlsx
+++ b/artifacts/cache-hit-budget.xlsx
@@ -13,24 +13,26 @@
     <sheet name="Volume" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Category totals" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Category usage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Profiles" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Scenarios" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Additional costs" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Pricing" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Read me" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Category costs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Profiles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Scenarios" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Additional costs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Read me" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculations'!$A$1:$AF$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculations'!$A$1:$AI$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agents'!$A$1:$N$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volume'!$A$1:$J$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Category totals'!$A$1:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category usage'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Profiles'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Pricing'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Read me'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category costs'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Profiles'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Pricing'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Read me'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -619,6 +621,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No items</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:A1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -716,7 +743,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01T17:17:40.416Z</t>
+          <t>2026-10-01T18:21:05.096Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -752,7 +779,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01T17:17:23.084029+00:00</t>
+          <t>2026-10-01T18:20:46.699392+00:00</t>
         </is>
       </c>
       <c r="I3" s="2" t="b">
@@ -767,13 +794,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -863,89 +890,101 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tier rates</t>
+          <t>Category token costs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
+          <t>Category costs splits Expected-scenario tokens into uncached input, cached reads, cache writes and output. Known costs sum the corresponding Calculations formulas. Blended USD/1M is derived from each token-type subtotal when pricing is complete; inspect Calculations for each model's selected rate. Incomplete rows omit unpriced agent lines from costs while retaining their token counts. Re-export after resolving pricing or limits.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Partial totals</t>
+          <t>Tier rates</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
+          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Annualization</t>
+          <t>Partial totals</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
+          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Annualization</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
+          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Scenarios</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
+          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Detailed workflows</t>
+          <t>Scenarios</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Detailed workflows</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Schema 2; defaults 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -956,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF10"/>
+  <dimension ref="A1:AI10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -991,6 +1030,9 @@
     <col width="33" customWidth="1" min="30" max="30"/>
     <col width="25" customWidth="1" min="31" max="31"/>
     <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="30" customWidth="1" min="33" max="33"/>
+    <col width="27" customWidth="1" min="34" max="34"/>
+    <col width="27" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1154,6 +1196,21 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Uncached input tokens/month</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Cached read tokens/month</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Cache write tokens/month</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1272,6 +1329,18 @@
           <t>simple</t>
         </is>
       </c>
+      <c r="AG2" s="2">
+        <f>R2*(1-K2-L2)</f>
+        <v/>
+      </c>
+      <c r="AH2" s="2">
+        <f>R2*K2</f>
+        <v/>
+      </c>
+      <c r="AI2" s="2">
+        <f>R2*L2</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1377,6 +1446,18 @@
           <t>medium</t>
         </is>
       </c>
+      <c r="AG3" s="2">
+        <f>R3*(1-K3-L3)</f>
+        <v/>
+      </c>
+      <c r="AH3" s="2">
+        <f>R3*K3</f>
+        <v/>
+      </c>
+      <c r="AI3" s="2">
+        <f>R3*L3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1482,6 +1563,18 @@
           <t>high</t>
         </is>
       </c>
+      <c r="AG4" s="2">
+        <f>R4*(1-K4-L4)</f>
+        <v/>
+      </c>
+      <c r="AH4" s="2">
+        <f>R4*K4</f>
+        <v/>
+      </c>
+      <c r="AI4" s="2">
+        <f>R4*L4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1600,6 +1693,18 @@
           <t>simple</t>
         </is>
       </c>
+      <c r="AG5" s="2">
+        <f>R5*(1-K5-L5)</f>
+        <v/>
+      </c>
+      <c r="AH5" s="2">
+        <f>R5*K5</f>
+        <v/>
+      </c>
+      <c r="AI5" s="2">
+        <f>R5*L5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1705,6 +1810,18 @@
           <t>medium</t>
         </is>
       </c>
+      <c r="AG6" s="2">
+        <f>R6*(1-K6-L6)</f>
+        <v/>
+      </c>
+      <c r="AH6" s="2">
+        <f>R6*K6</f>
+        <v/>
+      </c>
+      <c r="AI6" s="2">
+        <f>R6*L6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1810,6 +1927,18 @@
           <t>high</t>
         </is>
       </c>
+      <c r="AG7" s="2">
+        <f>R7*(1-K7-L7)</f>
+        <v/>
+      </c>
+      <c r="AH7" s="2">
+        <f>R7*K7</f>
+        <v/>
+      </c>
+      <c r="AI7" s="2">
+        <f>R7*L7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1928,6 +2057,18 @@
           <t>simple</t>
         </is>
       </c>
+      <c r="AG8" s="2">
+        <f>R8*(1-K8-L8)</f>
+        <v/>
+      </c>
+      <c r="AH8" s="2">
+        <f>R8*K8</f>
+        <v/>
+      </c>
+      <c r="AI8" s="2">
+        <f>R8*L8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2033,6 +2174,18 @@
           <t>medium</t>
         </is>
       </c>
+      <c r="AG9" s="2">
+        <f>R9*(1-K9-L9)</f>
+        <v/>
+      </c>
+      <c r="AH9" s="2">
+        <f>R9*K9</f>
+        <v/>
+      </c>
+      <c r="AI9" s="2">
+        <f>R9*L9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2138,9 +2291,21 @@
           <t>high</t>
         </is>
       </c>
+      <c r="AG10" s="2">
+        <f>R10*(1-K10-L10)</f>
+        <v/>
+      </c>
+      <c r="AH10" s="2">
+        <f>R10*K10</f>
+        <v/>
+      </c>
+      <c r="AI10" s="2">
+        <f>R10*L10</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF10"/>
+  <autoFilter ref="A1:AI10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2758,6 +2923,484 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Token type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens/month</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Known cost USD/month</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Blended USD/1M tokens</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Uncached input</t>
+        </is>
+      </c>
+      <c r="C2" s="2">
+        <f>SUMIFS(Calculations!AG2:AG10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A2)</f>
+        <v/>
+      </c>
+      <c r="D2" s="2">
+        <f>SUMIFS(Calculations!T2:T10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A2)</f>
+        <v/>
+      </c>
+      <c r="E2" s="2">
+        <f>IF(C2=0,"",D2*1000000/C2)</f>
+        <v/>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cached input read</t>
+        </is>
+      </c>
+      <c r="C3" s="2">
+        <f>SUMIFS(Calculations!AH2:AH10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A3)</f>
+        <v/>
+      </c>
+      <c r="D3" s="2">
+        <f>SUMIFS(Calculations!V2:V10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A3)</f>
+        <v/>
+      </c>
+      <c r="E3" s="2">
+        <f>IF(C3=0,"",D3*1000000/C3)</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Input cache write</t>
+        </is>
+      </c>
+      <c r="C4" s="2">
+        <f>SUMIFS(Calculations!AI2:AI10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A4)</f>
+        <v/>
+      </c>
+      <c r="D4" s="2">
+        <f>SUMIFS(Calculations!W2:W10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A4)</f>
+        <v/>
+      </c>
+      <c r="E4" s="2">
+        <f>IF(C4=0,"",D4*1000000/C4)</f>
+        <v/>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Output incl. reasoning</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <f>SUMIFS(Calculations!S2:S10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>SUMIFS(Calculations!U2:U10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="2">
+        <f>IF(C5=0,"",D5*1000000/C5)</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C6" s="2">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="2">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Uncached input</t>
+        </is>
+      </c>
+      <c r="C7" s="2">
+        <f>SUMIFS(Calculations!AG2:AG10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="2">
+        <f>SUMIFS(Calculations!T2:T10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="2">
+        <f>IF(C7=0,"",D7*1000000/C7)</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cached input read</t>
+        </is>
+      </c>
+      <c r="C8" s="2">
+        <f>SUMIFS(Calculations!AH2:AH10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="2">
+        <f>SUMIFS(Calculations!V2:V10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="2">
+        <f>IF(C8=0,"",D8*1000000/C8)</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Input cache write</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <f>SUMIFS(Calculations!AI2:AI10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="2">
+        <f>SUMIFS(Calculations!W2:W10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="2">
+        <f>IF(C9=0,"",D9*1000000/C9)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Output incl. reasoning</t>
+        </is>
+      </c>
+      <c r="C10" s="2">
+        <f>SUMIFS(Calculations!S2:S10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="2">
+        <f>SUMIFS(Calculations!U2:U10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="2">
+        <f>IF(C10=0,"",D10*1000000/C10)</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" s="2">
+        <f>SUM(C7:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="2">
+        <f>SUM(D7:D10)</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Uncached input</t>
+        </is>
+      </c>
+      <c r="C12" s="2">
+        <f>SUMIFS(Calculations!AG2:AG10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A12)</f>
+        <v/>
+      </c>
+      <c r="D12" s="2">
+        <f>SUMIFS(Calculations!T2:T10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="2">
+        <f>IF(C12=0,"",D12*1000000/C12)</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cached input read</t>
+        </is>
+      </c>
+      <c r="C13" s="2">
+        <f>SUMIFS(Calculations!AH2:AH10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A13)</f>
+        <v/>
+      </c>
+      <c r="D13" s="2">
+        <f>SUMIFS(Calculations!V2:V10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="2">
+        <f>IF(C13=0,"",D13*1000000/C13)</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Input cache write</t>
+        </is>
+      </c>
+      <c r="C14" s="2">
+        <f>SUMIFS(Calculations!AI2:AI10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="2">
+        <f>SUMIFS(Calculations!W2:W10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="2">
+        <f>IF(C14=0,"",D14*1000000/C14)</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Output incl. reasoning</t>
+        </is>
+      </c>
+      <c r="C15" s="2">
+        <f>SUMIFS(Calculations!S2:S10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A15)</f>
+        <v/>
+      </c>
+      <c r="D15" s="2">
+        <f>SUMIFS(Calculations!U2:U10,Calculations!A2:A10,"Expected",Calculations!AF2:AF10,A15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="2">
+        <f>IF(C15=0,"",D15*1000000/C15)</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C16" s="2">
+        <f>SUM(C12:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="2">
+        <f>SUM(D12:D15)</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2937,7 +3580,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3092,29 +3735,4 @@
   <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>No items</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:A1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Show daily and monthly category token costs
</commit_message>
<xml_diff>
--- a/artifacts/cache-hit-budget.xlsx
+++ b/artifacts/cache-hit-budget.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volume'!$A$1:$J$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Category totals'!$A$1:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category usage'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category costs'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category costs'!$A$1:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Profiles'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
@@ -743,7 +743,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01T18:21:05.096Z</t>
+          <t>2026-10-01T19:13:41.675Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -779,7 +779,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01T18:20:46.699392+00:00</t>
+          <t>2026-10-01T19:13:23.196497+00:00</t>
         </is>
       </c>
       <c r="I3" s="2" t="b">
@@ -895,7 +895,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Category costs splits Expected-scenario tokens into uncached input, cached reads, cache writes and output. Known costs sum the corresponding Calculations formulas. Blended USD/1M is derived from each token-type subtotal when pricing is complete; inspect Calculations for each model's selected rate. Incomplete rows omit unpriced agent lines from costs while retaining their token counts. Re-export after resolving pricing or limits.</t>
+          <t>Category costs splits Expected-scenario tokens into uncached input, cached reads, cache writes and output. Known monthly costs sum the corresponding Calculations formulas; average daily tokens and costs divide monthly values by 30 planning days. Blended USD/1M is derived from each token-type subtotal when pricing is complete; inspect Calculations for each model's selected rate. Incomplete rows omit unpriced agent lines from costs while retaining their token counts. Re-export after resolving pricing or limits.</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2932,6 +2932,9 @@
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2965,6 +2968,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Average tokens/day</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Known cost USD/day</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Planning days/month</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2994,6 +3012,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G2" s="2">
+        <f>C2/I2</f>
+        <v/>
+      </c>
+      <c r="H2" s="2">
+        <f>D2/I2</f>
+        <v/>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3023,6 +3052,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G3" s="2">
+        <f>C3/I3</f>
+        <v/>
+      </c>
+      <c r="H3" s="2">
+        <f>D3/I3</f>
+        <v/>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3052,6 +3092,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G4" s="2">
+        <f>C4/I4</f>
+        <v/>
+      </c>
+      <c r="H4" s="2">
+        <f>D4/I4</f>
+        <v/>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3081,6 +3132,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G5" s="2">
+        <f>C5/I5</f>
+        <v/>
+      </c>
+      <c r="H5" s="2">
+        <f>D5/I5</f>
+        <v/>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3106,6 +3168,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G6" s="2">
+        <f>C6/I6</f>
+        <v/>
+      </c>
+      <c r="H6" s="2">
+        <f>D6/I6</f>
+        <v/>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3135,6 +3208,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G7" s="2">
+        <f>C7/I7</f>
+        <v/>
+      </c>
+      <c r="H7" s="2">
+        <f>D7/I7</f>
+        <v/>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3164,6 +3248,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G8" s="2">
+        <f>C8/I8</f>
+        <v/>
+      </c>
+      <c r="H8" s="2">
+        <f>D8/I8</f>
+        <v/>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3193,6 +3288,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G9" s="2">
+        <f>C9/I9</f>
+        <v/>
+      </c>
+      <c r="H9" s="2">
+        <f>D9/I9</f>
+        <v/>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3222,6 +3328,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G10" s="2">
+        <f>C10/I10</f>
+        <v/>
+      </c>
+      <c r="H10" s="2">
+        <f>D10/I10</f>
+        <v/>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3247,6 +3364,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G11" s="2">
+        <f>C11/I11</f>
+        <v/>
+      </c>
+      <c r="H11" s="2">
+        <f>D11/I11</f>
+        <v/>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3276,6 +3404,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G12" s="2">
+        <f>C12/I12</f>
+        <v/>
+      </c>
+      <c r="H12" s="2">
+        <f>D12/I12</f>
+        <v/>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3305,6 +3444,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G13" s="2">
+        <f>C13/I13</f>
+        <v/>
+      </c>
+      <c r="H13" s="2">
+        <f>D13/I13</f>
+        <v/>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3334,6 +3484,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G14" s="2">
+        <f>C14/I14</f>
+        <v/>
+      </c>
+      <c r="H14" s="2">
+        <f>D14/I14</f>
+        <v/>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3363,6 +3524,17 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G15" s="2">
+        <f>C15/I15</f>
+        <v/>
+      </c>
+      <c r="H15" s="2">
+        <f>D15/I15</f>
+        <v/>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3388,9 +3560,20 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="G16" s="2">
+        <f>C16/I16</f>
+        <v/>
+      </c>
+      <c r="H16" s="2">
+        <f>D16/I16</f>
+        <v/>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Summarize monthly input and output by category
</commit_message>
<xml_diff>
--- a/artifacts/cache-hit-budget.xlsx
+++ b/artifacts/cache-hit-budget.xlsx
@@ -14,11 +14,12 @@
     <sheet name="Category totals" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Category usage" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Category costs" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Profiles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Scenarios" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Additional costs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Read me" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Monthly category summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Profiles" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Scenarios" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Additional costs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Pricing" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Read me" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$H$4</definedName>
@@ -28,11 +29,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Category totals'!$A$1:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category usage'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category costs'!$A$1:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Profiles'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Pricing'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Read me'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Monthly category summary'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Profiles'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Pricing'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Read me'!$A$1:$B$16</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -621,6 +623,163 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>volume_factor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>calls_factor</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>input_factor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>output_factor</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>retry_factor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>model_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -640,7 +799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -743,7 +902,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01T19:13:41.675Z</t>
+          <t>2026-10-01T20:02:36.558Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -779,7 +938,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01T19:13:23.196497+00:00</t>
+          <t>2026-10-01T20:02:18.139027+00:00</t>
         </is>
       </c>
       <c r="I3" s="2" t="b">
@@ -794,13 +953,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -902,89 +1061,101 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tier rates</t>
+          <t>Monthly category summary</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
+          <t>Monthly category summary combines Category usage input/output token counts with Category costs. Input cost includes uncached input, cached reads, and cache writes; output includes billable reasoning. The suite row sums category values and reconciles to the Expected LLM amount in Summary. Incomplete values include only fully priced agent lines.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Partial totals</t>
+          <t>Tier rates</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
+          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Annualization</t>
+          <t>Partial totals</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
+          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Annualization</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
+          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Scenarios</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
+          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Detailed workflows</t>
+          <t>Scenarios</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Detailed workflows</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Schema 2; defaults 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3584,6 +3755,217 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Input tokens/month</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Known input USD/month</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Output tokens/month</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Known output USD/month</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total tokens/month</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Known LLM USD/month</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <f>'Category usage'!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2">
+        <f>SUM('Category costs'!D2:D4)</f>
+        <v/>
+      </c>
+      <c r="D2" s="2">
+        <f>'Category usage'!C2</f>
+        <v/>
+      </c>
+      <c r="E2" s="2">
+        <f>'Category costs'!D5</f>
+        <v/>
+      </c>
+      <c r="F2" s="2">
+        <f>B2+D2</f>
+        <v/>
+      </c>
+      <c r="G2" s="2">
+        <f>C2+E2</f>
+        <v/>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <f>'Category usage'!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2">
+        <f>SUM('Category costs'!D7:D9)</f>
+        <v/>
+      </c>
+      <c r="D3" s="2">
+        <f>'Category usage'!C3</f>
+        <v/>
+      </c>
+      <c r="E3" s="2">
+        <f>'Category costs'!D10</f>
+        <v/>
+      </c>
+      <c r="F3" s="2">
+        <f>B3+D3</f>
+        <v/>
+      </c>
+      <c r="G3" s="2">
+        <f>C3+E3</f>
+        <v/>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <f>'Category usage'!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2">
+        <f>SUM('Category costs'!D12:D14)</f>
+        <v/>
+      </c>
+      <c r="D4" s="2">
+        <f>'Category usage'!C4</f>
+        <v/>
+      </c>
+      <c r="E4" s="2">
+        <f>'Category costs'!D15</f>
+        <v/>
+      </c>
+      <c r="F4" s="2">
+        <f>B4+D4</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>C4+E4</f>
+        <v/>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Suite total</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <f>SUM(B2:B4)</f>
+        <v/>
+      </c>
+      <c r="C5" s="2">
+        <f>SUM(C2:C4)</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>SUM(D2:D4)</f>
+        <v/>
+      </c>
+      <c r="E5" s="2">
+        <f>SUM(E2:E4)</f>
+        <v/>
+      </c>
+      <c r="F5" s="2">
+        <f>B5+D5</f>
+        <v/>
+      </c>
+      <c r="G5" s="2">
+        <f>C5+E5</f>
+        <v/>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3761,161 +4143,4 @@
   <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>volume_factor</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>calls_factor</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>input_factor</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>output_factor</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>retry_factor</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>model_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add cost driver sensitivity previews
</commit_message>
<xml_diff>
--- a/artifacts/cache-hit-budget.xlsx
+++ b/artifacts/cache-hit-budget.xlsx
@@ -902,7 +902,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01T20:02:36.558Z</t>
+          <t>2026-10-02T18:37:15.145Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -938,7 +938,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01T20:02:18.139027+00:00</t>
+          <t>2026-10-02T18:36:52.696988+00:00</t>
         </is>
       </c>
       <c r="I3" s="2" t="b">

</xml_diff>

<commit_message>
Model agent invocation links
</commit_message>
<xml_diff>
--- a/artifacts/cache-hit-budget.xlsx
+++ b/artifacts/cache-hit-budget.xlsx
@@ -11,30 +11,32 @@
     <sheet name="Calculations" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Agents" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Volume" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Category totals" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Category usage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Category costs" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Monthly category summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Profiles" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Scenarios" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Additional costs" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Pricing" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Read me" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Agent links" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Category totals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Category usage" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Category costs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Monthly category summary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Profiles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Scenarios" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Additional costs" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Pricing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Read me" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculations'!$A$1:$AI$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agents'!$A$1:$N$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volume'!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Category totals'!$A$1:$B$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category usage'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category costs'!$A$1:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Monthly category summary'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Profiles'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Pricing'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Read me'!$A$1:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volume'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agent links'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category totals'!$A$1:$B$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category usage'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Category costs'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Monthly category summary'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Profiles'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pricing'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Read me'!$A$1:$B$17</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -623,6 +625,191 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>complexity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>calls</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>retry_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>cache_fraction</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>cache_write_fraction</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>model_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>deepseek/deepseek-coder</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -774,7 +961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -799,7 +986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -902,7 +1089,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-02T18:37:15.145Z</t>
+          <t>2026-10-02T20:28:51.930Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -938,7 +1125,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-02T18:36:52.696988+00:00</t>
+          <t>2026-10-02T20:28:23.208693+00:00</t>
         </is>
       </c>
       <c r="I3" s="2" t="b">
@@ -953,13 +1140,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1018,7 +1205,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Edit numeric inputs in Calculations to recalculate costs. Column F derives scenario monthly volume from columns Z–AE; daily mode uses a 30-day planning month. Profiles, Scenarios, Agents and Pricing document the snapshot; editing those sheets does not propagate to Calculations.</t>
+          <t>Edit numeric inputs in Calculations to recalculate costs. For direct-volume rows, column F derives scenario monthly volume from columns Z–AE using a 30-day planning month. For derived rows, column F is the graph result precomputed by the app; edit links or upstream volume in the app and re-export. Profiles, Scenarios, Agents and Pricing document the snapshot; editing those sheets does not propagate to Calculations.</t>
         </is>
       </c>
     </row>
@@ -1030,132 +1217,144 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Volume derives baseline monthly invocations per agent and all agents from the exported inventory. Category totals sums the Volume sheet by complexity. These totals exclude scenario volume multipliers; Calculations contains scenario-effective volumes.</t>
+          <t>Volume derives direct baseline invocations and records app-precomputed derived invocations. Category totals sums the Volume sheet by complexity. These totals exclude scenario volume multipliers; Calculations contains scenario-effective volumes.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Category token usage</t>
+          <t>Agent links</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Category usage sums Expected-scenario input and output tokens from Calculations, including normal calls and extra attempts. Cached input is part of input usage, not an extra category; billable reasoning is included in output. Average daily tokens divide monthly totals by 30 planning days.</t>
+          <t>Agent links shows effective Low/Expected/High probability, fanout, and child contributions. Parent totals are precomputed in topological order by the app; changing edges or parent totals in this workbook does not update derived rows in Calculations or Volume. Re-export from the app for a revised graph. Derived rows in Agents cannot be reimported without rebuilding links in the app.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Category token costs</t>
+          <t>Category token usage</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Category costs splits Expected-scenario tokens into uncached input, cached reads, cache writes and output. Known monthly costs sum the corresponding Calculations formulas; average daily tokens and costs divide monthly values by 30 planning days. Blended USD/1M is derived from each token-type subtotal when pricing is complete; inspect Calculations for each model's selected rate. Incomplete rows omit unpriced agent lines from costs while retaining their token counts. Re-export after resolving pricing or limits.</t>
+          <t>Category usage sums Expected-scenario input and output tokens from Calculations, including normal calls and extra attempts. Cached input is part of input usage, not an extra category; billable reasoning is included in output. Average daily tokens divide monthly totals by 30 planning days.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Monthly category summary</t>
+          <t>Category token costs</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Monthly category summary combines Category usage input/output token counts with Category costs. Input cost includes uncached input, cached reads, and cache writes; output includes billable reasoning. The suite row sums category values and reconciles to the Expected LLM amount in Summary. Incomplete values include only fully priced agent lines.</t>
+          <t>Category costs splits Expected-scenario tokens into uncached input, cached reads, cache writes and output. Known monthly costs sum the corresponding Calculations formulas; average daily tokens and costs divide monthly values by 30 planning days. Blended USD/1M is derived from each token-type subtotal when pricing is complete; inspect Calculations for each model's selected rate. Incomplete rows omit unpriced agent lines from costs while retaining their token counts. Re-export after resolving pricing or limits.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tier rates</t>
+          <t>Monthly category summary</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
+          <t>Monthly category summary combines Category usage input/output token counts with Category costs. Input cost includes uncached input, cached reads, and cache writes; output includes billable reasoning. The suite row sums category values and reconciles to the Expected LLM amount in Summary. Incomplete values include only fully priced agent lines.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Partial totals</t>
+          <t>Tier rates</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
+          <t>Rates in Calculations are selected using the exported per-call input size. After crossing a tier threshold, update the applicable rates from Pricing or re-export from the app.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Annualization</t>
+          <t>Partial totals</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
+          <t>Incomplete rows have blank costs; summaries are known subtotals, not full budgets.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Annualization</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
+          <t>First year = 12 identical recurring months + one-time items. Additional monthly/one-time values in Summary are editable frozen inputs.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Scenarios</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
+          <t>Text tokens, including total billable reasoning in output. Cache writes use supplied rates. Tools, cache storage, multimodal charges require additional items/custom rates.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Detailed workflows</t>
+          <t>Scenarios</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+          <t>Planning assumptions, not statistical confidence intervals. Execution fields in Calculations are scenario-effective values.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Detailed workflows</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Each step appears in Calculations and replaces the aggregate. The Agents sheet is an aggregate import template, not a lossless backup of detailed steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Schema 2; defaults 1</t>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Schema 3; defaults 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2698,7 +2897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2711,6 +2910,8 @@
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="39" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2764,6 +2965,16 @@
           <t>Total monthly invocations all agents</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Agent row ID</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Previous direct volume source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2804,6 +3015,11 @@
         <f>C2*I2</f>
         <v/>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>cb006f9f-1f25-4567-84d9-d16399b006cf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2844,6 +3060,11 @@
         <f>C3*I3</f>
         <v/>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>f93151c5-288a-4154-8c44-2dde32237ca3</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2884,14 +3105,110 @@
         <f>C4*I4</f>
         <v/>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>09e1b37a-ecb4-46fa-8ec5-26f0982af94e</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Parent agent/group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Child agent/group</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Branch group</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger probability</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Child invocations per trigger</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Parent invocations/month (precomputed)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Child invocations/month</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Link ID</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Parent row ID</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Child row ID</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2955,7 +3272,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3088,7 +3405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3749,7 +4066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3958,189 +4275,4 @@
   <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>complexity</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>calls</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>input_tokens</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>output_tokens</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>retry_rate</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>cache_fraction</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>cache_write_fraction</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>model_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>simple</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>deepseek/deepseek-coder</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>15000</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>